<commit_message>
Bugfix: whole-cell placeholders with numeric values were rendered as strings
</commit_message>
<xml_diff>
--- a/examples/simple/template.xlsx
+++ b/examples/simple/template.xlsx
@@ -14,15 +14,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Report: {{ title }}</t>
-  </si>
-  <si>
-    <t>Year: {{ year }}</t>
-  </si>
-  <si>
-    <t>Status: {% if active %}Active{% else %}Inactive{% endif %}</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>Report:</t>
+  </si>
+  <si>
+    <t>{{ title }}</t>
+  </si>
+  <si>
+    <t>Year:</t>
+  </si>
+  <si>
+    <t>{{ year }}</t>
+  </si>
+  <si>
+    <t>Status:</t>
+  </si>
+  <si>
+    <t>{% if active %}Active{% else %}Inactive{% endif %}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price: </t>
   </si>
   <si>
     <t xml:space="preserve">Price (2x): </t>
@@ -336,22 +348,39 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B4" t="str">
+        <f>{{ price }}</f>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="str">
         <f>={{ price }}*2</f>
       </c>
     </row>

</xml_diff>